<commit_message>
regenerate sales data with realistic 5-10% YoY growth
Replaced random +/-25% variation with consistent 5-10% uplift
over same day prior year plus small daily noise. March YoY now
shows 4.5-8.8% growth across all stores.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sales/sales.xlsx
+++ b/data/sales/sales.xlsx
@@ -9799,1016 +9799,1016 @@
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>March 1, 2026</v>
+        <v>February 28, 2026</v>
       </c>
       <c r="B370">
-        <v>296.82</v>
+        <v>514.96</v>
       </c>
       <c r="C370">
-        <v>1077.71</v>
+        <v>2601.09</v>
       </c>
       <c r="D370">
-        <v>1682.64</v>
+        <v>2069.66</v>
       </c>
       <c r="E370">
-        <v>524.37</v>
+        <v>1166.96</v>
       </c>
       <c r="F370">
-        <v>1244.64</v>
+        <v>2779.91</v>
       </c>
       <c r="G370">
-        <v>1494.25</v>
+        <v>2340.82</v>
       </c>
       <c r="H370">
-        <v>6320.43</v>
+        <v>11473.4</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>March 2, 2026</v>
+        <v>March 1, 2026</v>
       </c>
       <c r="B371">
-        <v>400.86</v>
+        <v>439.2</v>
       </c>
       <c r="C371">
-        <v>2286.25</v>
+        <v>1491.48</v>
       </c>
       <c r="D371">
-        <v>1344.29</v>
+        <v>1358.25</v>
       </c>
       <c r="E371">
-        <v>604.02</v>
+        <v>485.26</v>
       </c>
       <c r="F371">
-        <v>1279.08</v>
+        <v>1587.67</v>
       </c>
       <c r="G371">
-        <v>1357.04</v>
+        <v>1622.75</v>
       </c>
       <c r="H371">
-        <v>7271.54</v>
+        <v>6984.61</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>March 3, 2026</v>
+        <v>March 2, 2026</v>
       </c>
       <c r="B372">
-        <v>533.17</v>
+        <v>553.16</v>
       </c>
       <c r="C372">
-        <v>1922.67</v>
+        <v>2007.43</v>
       </c>
       <c r="D372">
-        <v>1372.69</v>
+        <v>908.23</v>
       </c>
       <c r="E372">
-        <v>608.28</v>
+        <v>690.74</v>
       </c>
       <c r="F372">
-        <v>1420.48</v>
+        <v>1647.45</v>
       </c>
       <c r="G372">
-        <v>1591.56</v>
+        <v>1124.83</v>
       </c>
       <c r="H372">
-        <v>7448.85</v>
+        <v>6931.84</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>March 4, 2026</v>
+        <v>March 3, 2026</v>
       </c>
       <c r="B373">
-        <v>680.54</v>
+        <v>551.68</v>
       </c>
       <c r="C373">
-        <v>2523.34</v>
+        <v>2242.43</v>
       </c>
       <c r="D373">
-        <v>2492.49</v>
+        <v>1699.5</v>
       </c>
       <c r="E373">
-        <v>796.24</v>
+        <v>546.82</v>
       </c>
       <c r="F373">
-        <v>2326.64</v>
+        <v>1692.62</v>
       </c>
       <c r="G373">
-        <v>1943.87</v>
+        <v>1534.76</v>
       </c>
       <c r="H373">
-        <v>10763.12</v>
+        <v>8267.81</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>March 5, 2026</v>
+        <v>March 4, 2026</v>
       </c>
       <c r="B374">
-        <v>510.95</v>
+        <v>375.99</v>
       </c>
       <c r="C374">
-        <v>1842.94</v>
+        <v>2546.59</v>
       </c>
       <c r="D374">
-        <v>2165.25</v>
+        <v>2014.45</v>
       </c>
       <c r="E374">
-        <v>941.6</v>
+        <v>832.22</v>
       </c>
       <c r="F374">
-        <v>2107.57</v>
+        <v>2237.41</v>
       </c>
       <c r="G374">
-        <v>1216.09</v>
+        <v>763.27</v>
       </c>
       <c r="H374">
-        <v>8784.4</v>
+        <v>8769.93</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>March 6, 2026</v>
+        <v>March 5, 2026</v>
       </c>
       <c r="B375">
-        <v>1013.35</v>
+        <v>691.75</v>
       </c>
       <c r="C375">
-        <v>2081.08</v>
+        <v>2068.23</v>
       </c>
       <c r="D375">
-        <v>2018.73</v>
+        <v>1906.09</v>
       </c>
       <c r="E375">
-        <v>886.41</v>
+        <v>727.95</v>
       </c>
       <c r="F375">
-        <v>3191.11</v>
+        <v>2111.03</v>
       </c>
       <c r="G375">
-        <v>2719.05</v>
+        <v>1166.03</v>
       </c>
       <c r="H375">
-        <v>11909.73</v>
+        <v>8671.08</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>March 7, 2026</v>
+        <v>March 6, 2026</v>
       </c>
       <c r="B376">
-        <v>579.32</v>
+        <v>2855.7</v>
       </c>
       <c r="C376">
-        <v>2275.67</v>
+        <v>4585.87</v>
       </c>
       <c r="D376">
-        <v>1859.66</v>
+        <v>2020.16</v>
       </c>
       <c r="E376">
-        <v>886.99</v>
+        <v>1050.73</v>
       </c>
       <c r="F376">
-        <v>1857.11</v>
+        <v>2854.35</v>
       </c>
       <c r="G376">
-        <v>1840.67</v>
+        <v>2657.26</v>
       </c>
       <c r="H376">
-        <v>9299.42</v>
+        <v>16024.07</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>March 8, 2026</v>
+        <v>March 7, 2026</v>
       </c>
       <c r="B377">
-        <v>460.19</v>
+        <v>426.88</v>
       </c>
       <c r="C377">
-        <v>1670.03</v>
+        <v>1598.73</v>
       </c>
       <c r="D377">
-        <v>1298.17</v>
+        <v>2943.2</v>
       </c>
       <c r="E377">
-        <v>332.95</v>
+        <v>746.29</v>
       </c>
       <c r="F377">
-        <v>1284.76</v>
+        <v>2283.84</v>
       </c>
       <c r="G377">
-        <v>1500.34</v>
+        <v>2393.99</v>
       </c>
       <c r="H377">
-        <v>6546.44</v>
+        <v>10392.93</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>March 9, 2026</v>
+        <v>March 8, 2026</v>
       </c>
       <c r="B378">
-        <v>389.39</v>
+        <v>489.23</v>
       </c>
       <c r="C378">
-        <v>1894.66</v>
+        <v>1367.08</v>
       </c>
       <c r="D378">
-        <v>1527.36</v>
+        <v>1057.85</v>
       </c>
       <c r="E378">
-        <v>578.15</v>
+        <v>668.18</v>
       </c>
       <c r="F378">
-        <v>1974.49</v>
+        <v>1286.03</v>
       </c>
       <c r="G378">
-        <v>1235.13</v>
+        <v>1074.44</v>
       </c>
       <c r="H378">
-        <v>7599.18</v>
+        <v>5942.81</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>March 10, 2026</v>
+        <v>March 9, 2026</v>
       </c>
       <c r="B379">
-        <v>392.38</v>
+        <v>461.74</v>
       </c>
       <c r="C379">
-        <v>2177.73</v>
+        <v>1314.16</v>
       </c>
       <c r="D379">
-        <v>1876.28</v>
+        <v>981.99</v>
       </c>
       <c r="E379">
-        <v>589.66</v>
+        <v>670.23</v>
       </c>
       <c r="F379">
-        <v>2035.63</v>
+        <v>1357.29</v>
       </c>
       <c r="G379">
-        <v>1269.9</v>
+        <v>1101.86</v>
       </c>
       <c r="H379">
-        <v>8341.58</v>
+        <v>5887.27</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>March 11, 2026</v>
+        <v>March 10, 2026</v>
       </c>
       <c r="B380">
-        <v>712.38</v>
+        <v>593.15</v>
       </c>
       <c r="C380">
-        <v>1825.94</v>
+        <v>1435.93</v>
       </c>
       <c r="D380">
-        <v>1879.45</v>
+        <v>1288.22</v>
       </c>
       <c r="E380">
-        <v>746.91</v>
+        <v>691.56</v>
       </c>
       <c r="F380">
-        <v>2014.93</v>
+        <v>1409</v>
       </c>
       <c r="G380">
-        <v>1330.26</v>
+        <v>887.63</v>
       </c>
       <c r="H380">
-        <v>8509.87</v>
+        <v>6305.49</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>March 12, 2026</v>
+        <v>March 11, 2026</v>
       </c>
       <c r="B381">
-        <v>472.84</v>
+        <v>473.09</v>
       </c>
       <c r="C381">
-        <v>2145.18</v>
+        <v>1748.08</v>
       </c>
       <c r="D381">
-        <v>1992.1</v>
+        <v>1333.21</v>
       </c>
       <c r="E381">
-        <v>752.91</v>
+        <v>935.58</v>
       </c>
       <c r="F381">
-        <v>1749.13</v>
+        <v>806.79</v>
       </c>
       <c r="G381">
-        <v>1585.73</v>
+        <v>928.36</v>
       </c>
       <c r="H381">
-        <v>8697.89</v>
+        <v>6225.11</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>March 13, 2026</v>
+        <v>March 12, 2026</v>
       </c>
       <c r="B382">
-        <v>1150.64</v>
+        <v>509.71</v>
       </c>
       <c r="C382">
-        <v>2353.56</v>
+        <v>1889.08</v>
       </c>
       <c r="D382">
-        <v>3139.87</v>
+        <v>1282.55</v>
       </c>
       <c r="E382">
-        <v>1010.81</v>
+        <v>738.81</v>
       </c>
       <c r="F382">
-        <v>2498.15</v>
+        <v>2031.35</v>
       </c>
       <c r="G382">
-        <v>2204.11</v>
+        <v>1154.55</v>
       </c>
       <c r="H382">
-        <v>12357.14</v>
+        <v>7606.05</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>March 14, 2026</v>
+        <v>March 13, 2026</v>
       </c>
       <c r="B383">
-        <v>404.3</v>
+        <v>1918</v>
       </c>
       <c r="C383">
-        <v>2140.7</v>
+        <v>2043.96</v>
       </c>
       <c r="D383">
-        <v>2511.21</v>
+        <v>1519.17</v>
       </c>
       <c r="E383">
-        <v>884.36</v>
+        <v>976.86</v>
       </c>
       <c r="F383">
-        <v>2102.47</v>
+        <v>2381.57</v>
       </c>
       <c r="G383">
-        <v>2207.46</v>
+        <v>1356.72</v>
       </c>
       <c r="H383">
-        <v>10250.5</v>
+        <v>10196.28</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>March 15, 2026</v>
+        <v>March 14, 2026</v>
       </c>
       <c r="B384">
-        <v>381.68</v>
+        <v>791.41</v>
       </c>
       <c r="C384">
-        <v>1444.72</v>
+        <v>3303.19</v>
       </c>
       <c r="D384">
-        <v>1757.79</v>
+        <v>2315.98</v>
       </c>
       <c r="E384">
-        <v>463.87</v>
+        <v>1235.65</v>
       </c>
       <c r="F384">
-        <v>1437.79</v>
+        <v>3065.07</v>
       </c>
       <c r="G384">
-        <v>1427.21</v>
+        <v>2840.84</v>
       </c>
       <c r="H384">
-        <v>6913.06</v>
+        <v>13552.14</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>March 16, 2026</v>
+        <v>March 15, 2026</v>
       </c>
       <c r="B385">
-        <v>411.1</v>
+        <v>677.72</v>
       </c>
       <c r="C385">
-        <v>2057.48</v>
+        <v>2349.55</v>
       </c>
       <c r="D385">
-        <v>1695.66</v>
+        <v>1578.95</v>
       </c>
       <c r="E385">
-        <v>589.12</v>
+        <v>1020.98</v>
       </c>
       <c r="F385">
-        <v>1406.3</v>
+        <v>2208.58</v>
       </c>
       <c r="G385">
-        <v>1087.31</v>
+        <v>1881.46</v>
       </c>
       <c r="H385">
-        <v>7246.97</v>
+        <v>9717.24</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>March 17, 2026</v>
+        <v>March 16, 2026</v>
       </c>
       <c r="B386">
-        <v>432.98</v>
+        <v>402.39</v>
       </c>
       <c r="C386">
-        <v>1689.83</v>
+        <v>1120.24</v>
       </c>
       <c r="D386">
-        <v>1217.48</v>
+        <v>1192.15</v>
       </c>
       <c r="E386">
-        <v>786.2</v>
+        <v>571.4</v>
       </c>
       <c r="F386">
-        <v>1743.14</v>
+        <v>1152.69</v>
       </c>
       <c r="G386">
-        <v>1734.94</v>
+        <v>925.07</v>
       </c>
       <c r="H386">
-        <v>7604.57</v>
+        <v>5363.94</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>March 18, 2026</v>
+        <v>March 17, 2026</v>
       </c>
       <c r="B387">
-        <v>733.08</v>
+        <v>446.78</v>
       </c>
       <c r="C387">
-        <v>2820.34</v>
+        <v>1289.03</v>
       </c>
       <c r="D387">
-        <v>1875.58</v>
+        <v>1097.28</v>
       </c>
       <c r="E387">
-        <v>554.53</v>
+        <v>598.6</v>
       </c>
       <c r="F387">
-        <v>2170.54</v>
+        <v>1553.42</v>
       </c>
       <c r="G387">
-        <v>1828.81</v>
+        <v>1446.75</v>
       </c>
       <c r="H387">
-        <v>9982.88</v>
+        <v>6431.86</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>March 19, 2026</v>
+        <v>March 18, 2026</v>
       </c>
       <c r="B388">
-        <v>701.16</v>
+        <v>632.3</v>
       </c>
       <c r="C388">
-        <v>2008.68</v>
+        <v>1870.95</v>
       </c>
       <c r="D388">
-        <v>2214.03</v>
+        <v>1286.81</v>
       </c>
       <c r="E388">
-        <v>624.57</v>
+        <v>709.39</v>
       </c>
       <c r="F388">
-        <v>2355.02</v>
+        <v>2208.5</v>
       </c>
       <c r="G388">
-        <v>1743.95</v>
+        <v>902.19</v>
       </c>
       <c r="H388">
-        <v>9647.41</v>
+        <v>7610.14</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>March 20, 2026</v>
+        <v>March 19, 2026</v>
       </c>
       <c r="B389">
-        <v>1139.4</v>
+        <v>1914.72</v>
       </c>
       <c r="C389">
-        <v>3121.98</v>
+        <v>2914.5</v>
       </c>
       <c r="D389">
-        <v>2550.68</v>
+        <v>1594.3</v>
       </c>
       <c r="E389">
-        <v>1105.7</v>
+        <v>848.31</v>
       </c>
       <c r="F389">
-        <v>2051.24</v>
+        <v>1578.22</v>
       </c>
       <c r="G389">
-        <v>1693.51</v>
+        <v>1688.81</v>
       </c>
       <c r="H389">
-        <v>11662.51</v>
+        <v>10538.86</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>March 21, 2026</v>
+        <v>March 20, 2026</v>
       </c>
       <c r="B390">
-        <v>465.8</v>
+        <v>533.49</v>
       </c>
       <c r="C390">
-        <v>1732.63</v>
+        <v>2202.12</v>
       </c>
       <c r="D390">
-        <v>2144.8</v>
+        <v>2043.01</v>
       </c>
       <c r="E390">
-        <v>757.17</v>
+        <v>920.58</v>
       </c>
       <c r="F390">
-        <v>2492.57</v>
+        <v>1121.87</v>
       </c>
       <c r="G390">
-        <v>1763.94</v>
+        <v>1605.08</v>
       </c>
       <c r="H390">
-        <v>9356.91</v>
+        <v>8426.15</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>March 22, 2026</v>
+        <v>March 21, 2026</v>
       </c>
       <c r="B391">
-        <v>339.05</v>
+        <v>691.47</v>
       </c>
       <c r="C391">
-        <v>1603.17</v>
+        <v>3175.17</v>
       </c>
       <c r="D391">
-        <v>1115.69</v>
+        <v>2274.65</v>
       </c>
       <c r="E391">
-        <v>386.54</v>
+        <v>1310.84</v>
       </c>
       <c r="F391">
-        <v>1551.73</v>
+        <v>2599.33</v>
       </c>
       <c r="G391">
-        <v>1038.12</v>
+        <v>1758.79</v>
       </c>
       <c r="H391">
-        <v>6034.3</v>
+        <v>11810.25</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>March 23, 2026</v>
+        <v>March 22, 2026</v>
       </c>
       <c r="B392">
-        <v>427.39</v>
+        <v>444.58</v>
       </c>
       <c r="C392">
-        <v>1655.4</v>
+        <v>1564.14</v>
       </c>
       <c r="D392">
-        <v>1142.32</v>
+        <v>2160.05</v>
       </c>
       <c r="E392">
-        <v>645.9</v>
+        <v>1028.91</v>
       </c>
       <c r="F392">
-        <v>1955.66</v>
+        <v>1704.61</v>
       </c>
       <c r="G392">
-        <v>1272.77</v>
+        <v>1940.34</v>
       </c>
       <c r="H392">
-        <v>7099.44</v>
+        <v>8842.63</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>March 24, 2026</v>
+        <v>March 23, 2026</v>
       </c>
       <c r="B393">
-        <v>598.83</v>
+        <v>662.7</v>
       </c>
       <c r="C393">
-        <v>2349.53</v>
+        <v>1210.26</v>
       </c>
       <c r="D393">
-        <v>1919.97</v>
+        <v>905.12</v>
       </c>
       <c r="E393">
-        <v>541.3</v>
+        <v>492.97</v>
       </c>
       <c r="F393">
-        <v>1771.66</v>
+        <v>1093.23</v>
       </c>
       <c r="G393">
-        <v>1441.23</v>
+        <v>1027.06</v>
       </c>
       <c r="H393">
-        <v>8622.52</v>
+        <v>5391.34</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>March 25, 2026</v>
+        <v>March 24, 2026</v>
       </c>
       <c r="B394">
-        <v>520.22</v>
+        <v>554.96</v>
       </c>
       <c r="C394">
-        <v>1898.51</v>
+        <v>2225.13</v>
       </c>
       <c r="D394">
-        <v>1897.81</v>
+        <v>1181.48</v>
       </c>
       <c r="E394">
-        <v>847.03</v>
+        <v>512.59</v>
       </c>
       <c r="F394">
-        <v>2344.79</v>
+        <v>1108.72</v>
       </c>
       <c r="G394">
-        <v>1337.28</v>
+        <v>796.27</v>
       </c>
       <c r="H394">
-        <v>8845.64</v>
+        <v>6379.15</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>March 26, 2026</v>
+        <v>March 25, 2026</v>
       </c>
       <c r="B395">
-        <v>519.57</v>
+        <v>942.23</v>
       </c>
       <c r="C395">
-        <v>2451.9</v>
+        <v>2048.56</v>
       </c>
       <c r="D395">
-        <v>1846.87</v>
+        <v>2057.14</v>
       </c>
       <c r="E395">
-        <v>788.41</v>
+        <v>696.93</v>
       </c>
       <c r="F395">
-        <v>1769.41</v>
+        <v>1743.9</v>
       </c>
       <c r="G395">
-        <v>1610.15</v>
+        <v>1290.85</v>
       </c>
       <c r="H395">
-        <v>8986.31</v>
+        <v>8779.61</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>March 27, 2026</v>
+        <v>March 26, 2026</v>
       </c>
       <c r="B396">
-        <v>1036.06</v>
+        <v>477.14</v>
       </c>
       <c r="C396">
-        <v>2571.12</v>
+        <v>2541.88</v>
       </c>
       <c r="D396">
-        <v>2877.39</v>
+        <v>1546.12</v>
       </c>
       <c r="E396">
-        <v>694.91</v>
+        <v>974.1</v>
       </c>
       <c r="F396">
-        <v>3000.23</v>
+        <v>1976.14</v>
       </c>
       <c r="G396">
-        <v>2496.3</v>
+        <v>1332.37</v>
       </c>
       <c r="H396">
-        <v>12676.01</v>
+        <v>8847.75</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>March 28, 2026</v>
+        <v>March 27, 2026</v>
       </c>
       <c r="B397">
-        <v>455.67</v>
+        <v>590.35</v>
       </c>
       <c r="C397">
-        <v>1918.97</v>
+        <v>1941.33</v>
       </c>
       <c r="D397">
-        <v>2169.69</v>
+        <v>1401.23</v>
       </c>
       <c r="E397">
-        <v>641.3</v>
+        <v>1202.48</v>
       </c>
       <c r="F397">
-        <v>1797.8</v>
+        <v>2072.78</v>
       </c>
       <c r="G397">
-        <v>2468.87</v>
+        <v>1368.69</v>
       </c>
       <c r="H397">
-        <v>9452.3</v>
+        <v>8576.86</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>March 29, 2026</v>
+        <v>March 28, 2026</v>
       </c>
       <c r="B398">
-        <v>448.74</v>
+        <v>1038.73</v>
       </c>
       <c r="C398">
-        <v>1390.71</v>
+        <v>3229.24</v>
       </c>
       <c r="D398">
-        <v>1753.11</v>
+        <v>2981.17</v>
       </c>
       <c r="E398">
-        <v>516.53</v>
+        <v>1171.76</v>
       </c>
       <c r="F398">
-        <v>1432.06</v>
+        <v>3432.13</v>
       </c>
       <c r="G398">
-        <v>1511.8</v>
+        <v>2517.79</v>
       </c>
       <c r="H398">
-        <v>7052.95</v>
+        <v>14370.82</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>March 30, 2026</v>
+        <v>March 29, 2026</v>
       </c>
       <c r="B399">
-        <v>374.98</v>
+        <v>556.78</v>
       </c>
       <c r="C399">
-        <v>1826.26</v>
+        <v>2527.88</v>
       </c>
       <c r="D399">
-        <v>1578.12</v>
+        <v>2547.49</v>
       </c>
       <c r="E399">
-        <v>565.96</v>
+        <v>933.05</v>
       </c>
       <c r="F399">
-        <v>1298.1</v>
+        <v>2296.92</v>
       </c>
       <c r="G399">
-        <v>1418.05</v>
+        <v>3056.69</v>
       </c>
       <c r="H399">
-        <v>7061.47</v>
+        <v>11918.81</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>March 31, 2026</v>
+        <v>March 30, 2026</v>
       </c>
       <c r="B400">
-        <v>582.61</v>
+        <v>374.7</v>
       </c>
       <c r="C400">
-        <v>2112.09</v>
+        <v>1647.75</v>
       </c>
       <c r="D400">
-        <v>1240.08</v>
+        <v>1552.23</v>
       </c>
       <c r="E400">
-        <v>546.89</v>
+        <v>517.73</v>
       </c>
       <c r="F400">
-        <v>1467.93</v>
+        <v>957.07</v>
       </c>
       <c r="G400">
-        <v>1151.05</v>
+        <v>1562.15</v>
       </c>
       <c r="H400">
-        <v>7100.65</v>
+        <v>6611.63</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>April 1, 2026</v>
+        <v>March 31, 2026</v>
       </c>
       <c r="B401">
-        <v>710.04</v>
+        <v>615.49</v>
       </c>
       <c r="C401">
-        <v>2287.18</v>
+        <v>2128.25</v>
       </c>
       <c r="D401">
-        <v>2025.7</v>
+        <v>1381.07</v>
       </c>
       <c r="E401">
-        <v>712.57</v>
+        <v>792.7</v>
       </c>
       <c r="F401">
-        <v>1694.62</v>
+        <v>1237.07</v>
       </c>
       <c r="G401">
-        <v>1638.61</v>
+        <v>1054.96</v>
       </c>
       <c r="H401">
-        <v>9068.72</v>
+        <v>7209.54</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>April 2, 2026</v>
+        <v>April 1, 2026</v>
       </c>
       <c r="B402">
-        <v>557.49</v>
+        <v>560.35</v>
       </c>
       <c r="C402">
-        <v>1718.62</v>
+        <v>2037.97</v>
       </c>
       <c r="D402">
-        <v>1899.77</v>
+        <v>1777.76</v>
       </c>
       <c r="E402">
-        <v>582.4</v>
+        <v>726.17</v>
       </c>
       <c r="F402">
-        <v>2007.3</v>
+        <v>1779.35</v>
       </c>
       <c r="G402">
-        <v>1165.1</v>
+        <v>1269.58</v>
       </c>
       <c r="H402">
-        <v>7930.68</v>
+        <v>8151.18</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>April 3, 2026</v>
+        <v>April 2, 2026</v>
       </c>
       <c r="B403">
-        <v>1265.03</v>
+        <v>602.75</v>
       </c>
       <c r="C403">
-        <v>2753.34</v>
+        <v>2916.39</v>
       </c>
       <c r="D403">
-        <v>2105.74</v>
+        <v>1842.25</v>
       </c>
       <c r="E403">
-        <v>995.75</v>
+        <v>729.68</v>
       </c>
       <c r="F403">
-        <v>2565.89</v>
+        <v>1824.14</v>
       </c>
       <c r="G403">
-        <v>1766.06</v>
+        <v>1528.8</v>
       </c>
       <c r="H403">
-        <v>11451.81</v>
+        <v>9444.01</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>April 4, 2026</v>
+        <v>April 3, 2026</v>
       </c>
       <c r="B404">
-        <v>501.96</v>
+        <v>526.84</v>
       </c>
       <c r="C404">
-        <v>1803.96</v>
+        <v>2530.81</v>
       </c>
       <c r="D404">
-        <v>1891.31</v>
+        <v>1670.81</v>
       </c>
       <c r="E404">
-        <v>841.89</v>
+        <v>966.72</v>
       </c>
       <c r="F404">
-        <v>1631.82</v>
+        <v>1677.98</v>
       </c>
       <c r="G404">
-        <v>2493.59</v>
+        <v>1597.77</v>
       </c>
       <c r="H404">
-        <v>9164.53</v>
+        <v>8970.93</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>April 5, 2026</v>
+        <v>April 4, 2026</v>
       </c>
       <c r="B405">
-        <v>363.65</v>
+        <v>833.21</v>
       </c>
       <c r="C405">
-        <v>1087.24</v>
+        <v>4520.52</v>
       </c>
       <c r="D405">
-        <v>1375.03</v>
+        <v>2403.5</v>
       </c>
       <c r="E405">
-        <v>360.94</v>
+        <v>1182.23</v>
       </c>
       <c r="F405">
-        <v>1000.69</v>
+        <v>3181.48</v>
       </c>
       <c r="G405">
-        <v>1189.68</v>
+        <v>2119.81</v>
       </c>
       <c r="H405">
-        <v>5377.23</v>
+        <v>14240.75</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>April 6, 2026</v>
+        <v>April 5, 2026</v>
       </c>
       <c r="B406">
-        <v>532.25</v>
+        <v>389.73</v>
       </c>
       <c r="C406">
-        <v>2042.84</v>
+        <v>2055.49</v>
       </c>
       <c r="D406">
-        <v>1545.45</v>
+        <v>2037.14</v>
       </c>
       <c r="E406">
-        <v>492.28</v>
+        <v>718.99</v>
       </c>
       <c r="F406">
-        <v>1248.96</v>
+        <v>2085.56</v>
       </c>
       <c r="G406">
-        <v>1390.49</v>
+        <v>1674.52</v>
       </c>
       <c r="H406">
-        <v>7252.27</v>
+        <v>8961.43</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>April 7, 2026</v>
+        <v>April 6, 2026</v>
       </c>
       <c r="B407">
-        <v>603.05</v>
+        <v>469.08</v>
       </c>
       <c r="C407">
-        <v>2053.17</v>
+        <v>1660.07</v>
       </c>
       <c r="D407">
-        <v>1378.09</v>
+        <v>942.24</v>
       </c>
       <c r="E407">
-        <v>535.19</v>
+        <v>418.78</v>
       </c>
       <c r="F407">
-        <v>1519.15</v>
+        <v>1676.86</v>
       </c>
       <c r="G407">
-        <v>1769.92</v>
+        <v>1488.71</v>
       </c>
       <c r="H407">
-        <v>7858.57</v>
+        <v>6655.74</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>April 8, 2026</v>
+        <v>April 7, 2026</v>
       </c>
       <c r="B408">
-        <v>725.59</v>
+        <v>484.98</v>
       </c>
       <c r="C408">
-        <v>2504.5</v>
+        <v>2361.88</v>
       </c>
       <c r="D408">
-        <v>1682.35</v>
+        <v>715.38</v>
       </c>
       <c r="E408">
-        <v>805.83</v>
+        <v>426.46</v>
       </c>
       <c r="F408">
-        <v>2227.28</v>
+        <v>1490.38</v>
       </c>
       <c r="G408">
-        <v>2027.89</v>
+        <v>1080.92</v>
       </c>
       <c r="H408">
-        <v>9973.44</v>
+        <v>6560</v>
       </c>
     </row>
     <row r="409">
@@ -10816,25 +10816,25 @@
         <v>Grand Total</v>
       </c>
       <c r="B409">
-        <v>242068.51</v>
+        <v>246313.12</v>
       </c>
       <c r="C409">
-        <v>847996.89</v>
+        <v>855187.7</v>
       </c>
       <c r="D409">
-        <v>764750.5</v>
+        <v>757557.64</v>
       </c>
       <c r="E409">
-        <v>273281.33</v>
+        <v>278391.08</v>
       </c>
       <c r="F409">
-        <v>778072.14</v>
+        <v>778336.58</v>
       </c>
       <c r="G409">
-        <v>663841.63</v>
+        <v>659743.08</v>
       </c>
       <c r="H409">
-        <v>3570011</v>
+        <v>3575529.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>